<commit_message>
Complete ecommerce backend CMS, category hierarchy, media, checkout, and docs
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/src/templates/product-import-template.xlsx
+++ b/src/templates/product-import-template.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC5"/>
+  <dimension ref="A1:AF5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -426,69 +426,75 @@
         <v>category</v>
       </c>
       <c r="H1" t="str">
-        <v>brand</v>
+        <v>main_category</v>
       </c>
       <c r="I1" t="str">
+        <v>sub_category</v>
+      </c>
+      <c r="J1" t="str">
+        <v>child_category</v>
+      </c>
+      <c r="L1" t="str">
         <v>unit_type</v>
       </c>
-      <c r="J1" t="str">
+      <c r="M1" t="str">
         <v>status</v>
       </c>
-      <c r="K1" t="str">
+      <c r="N1" t="str">
         <v>short_description</v>
       </c>
-      <c r="L1" t="str">
+      <c r="O1" t="str">
         <v>description</v>
       </c>
-      <c r="M1" t="str">
+      <c r="P1" t="str">
         <v>price</v>
       </c>
-      <c r="N1" t="str">
+      <c r="Q1" t="str">
         <v>sale_price</v>
       </c>
-      <c r="O1" t="str">
+      <c r="R1" t="str">
         <v>stock</v>
       </c>
-      <c r="P1" t="str">
+      <c r="S1" t="str">
         <v>featured_image</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="T1" t="str">
         <v>gallery_images</v>
       </c>
-      <c r="R1" t="str">
+      <c r="U1" t="str">
         <v>attribute_1_name</v>
       </c>
-      <c r="S1" t="str">
+      <c r="V1" t="str">
         <v>attribute_1_value</v>
       </c>
-      <c r="T1" t="str">
+      <c r="W1" t="str">
         <v>attribute_2_name</v>
       </c>
-      <c r="U1" t="str">
+      <c r="X1" t="str">
         <v>attribute_2_value</v>
       </c>
-      <c r="V1" t="str">
+      <c r="Y1" t="str">
         <v>variation_options</v>
       </c>
-      <c r="W1" t="str">
+      <c r="Z1" t="str">
         <v>seo_title</v>
       </c>
-      <c r="X1" t="str">
+      <c r="AA1" t="str">
         <v>seo_description</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="AB1" t="str">
         <v>tags</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AC1" t="str">
         <v>weight</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AD1" t="str">
         <v>length</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AE1" t="str">
         <v>width</v>
       </c>
-      <c r="AC1" t="str">
+      <c r="AF1" t="str">
         <v>height</v>
       </c>
     </row>
@@ -515,44 +521,44 @@
         <v>Apparel &gt; Tees</v>
       </c>
       <c r="H2" t="str">
-        <v>Acme Brand</v>
+        <v/>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
         <v>piece</v>
       </c>
-      <c r="J2" t="str">
+      <c r="M2" t="str">
         <v>published</v>
       </c>
-      <c r="K2" t="str">
+      <c r="N2" t="str">
         <v>Soft cotton everyday tee.</v>
       </c>
-      <c r="L2" t="str">
+      <c r="O2" t="str">
         <v>Comfortable crew neck tee for daily wear.</v>
       </c>
-      <c r="M2" t="str">
+      <c r="P2" t="str">
         <v>29.99</v>
       </c>
-      <c r="N2" t="str">
+      <c r="Q2" t="str">
         <v>24.99</v>
       </c>
-      <c r="O2" t="str">
+      <c r="R2" t="str">
         <v>100</v>
       </c>
-      <c r="P2" t="str">
+      <c r="S2" t="str">
         <v>https://cdn.example.com/tee-001.jpg</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="T2" t="str">
         <v>https://cdn.example.com/tee-001-a.jpg|https://cdn.example.com/tee-001-b.jpg</v>
       </c>
-      <c r="R2" t="str">
-        <v/>
-      </c>
-      <c r="S2" t="str">
-        <v/>
-      </c>
-      <c r="T2" t="str">
-        <v/>
-      </c>
       <c r="U2" t="str">
         <v/>
       </c>
@@ -560,24 +566,33 @@
         <v/>
       </c>
       <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
+        <v/>
+      </c>
+      <c r="Z2" t="str">
         <v>Classic Cotton Tee | Acme Store</v>
       </c>
-      <c r="X2" t="str">
+      <c r="AA2" t="str">
         <v>Shop our classic cotton tee.</v>
       </c>
-      <c r="Y2" t="str">
+      <c r="AB2" t="str">
         <v>tee,cotton,basics</v>
       </c>
-      <c r="Z2" t="str">
+      <c r="AC2" t="str">
         <v>0.25</v>
       </c>
-      <c r="AA2" t="str">
+      <c r="AD2" t="str">
         <v>30</v>
       </c>
-      <c r="AB2" t="str">
+      <c r="AE2" t="str">
         <v>25</v>
       </c>
-      <c r="AC2" t="str">
+      <c r="AF2" t="str">
         <v>2</v>
       </c>
     </row>
@@ -604,69 +619,78 @@
         <v>Apparel &gt; Hoodies</v>
       </c>
       <c r="H3" t="str">
-        <v>Acme Brand</v>
+        <v/>
       </c>
       <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
         <v>piece</v>
       </c>
-      <c r="J3" t="str">
+      <c r="M3" t="str">
         <v>published</v>
       </c>
-      <c r="K3" t="str">
+      <c r="N3" t="str">
         <v>Warm layered hoodie.</v>
       </c>
-      <c r="L3" t="str">
+      <c r="O3" t="str">
         <v>Premium fleece hoodie with kangaroo pocket.</v>
       </c>
-      <c r="M3" t="str">
+      <c r="P3" t="str">
         <v>59.99</v>
       </c>
-      <c r="N3" t="str">
-        <v/>
-      </c>
-      <c r="O3" t="str">
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
         <v>0</v>
       </c>
-      <c r="P3" t="str">
+      <c r="S3" t="str">
         <v>https://cdn.example.com/hd-100.jpg</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="T3" t="str">
         <v>https://cdn.example.com/hd-100-alt.jpg</v>
       </c>
-      <c r="R3" t="str">
+      <c r="U3" t="str">
         <v>Color</v>
       </c>
-      <c r="S3" t="str">
-        <v/>
-      </c>
-      <c r="T3" t="str">
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
         <v>Size</v>
       </c>
-      <c r="U3" t="str">
-        <v/>
-      </c>
-      <c r="V3" t="str">
+      <c r="X3" t="str">
+        <v/>
+      </c>
+      <c r="Y3" t="str">
         <v>Color;Size</v>
       </c>
-      <c r="W3" t="str">
+      <c r="Z3" t="str">
         <v>Hooded Sweatshirt</v>
       </c>
-      <c r="X3" t="str">
+      <c r="AA3" t="str">
         <v>Variable product parent row.</v>
       </c>
-      <c r="Y3" t="str">
+      <c r="AB3" t="str">
         <v>hoodie,apparel</v>
       </c>
-      <c r="Z3" t="str">
-        <v/>
-      </c>
-      <c r="AA3" t="str">
-        <v/>
-      </c>
-      <c r="AB3" t="str">
-        <v/>
-      </c>
       <c r="AC3" t="str">
+        <v/>
+      </c>
+      <c r="AD3" t="str">
+        <v/>
+      </c>
+      <c r="AE3" t="str">
+        <v/>
+      </c>
+      <c r="AF3" t="str">
         <v/>
       </c>
     </row>
@@ -699,63 +723,72 @@
         <v/>
       </c>
       <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
         <v>published</v>
       </c>
-      <c r="K4" t="str">
-        <v/>
-      </c>
-      <c r="L4" t="str">
-        <v/>
-      </c>
-      <c r="M4" t="str">
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
         <v>59.99</v>
       </c>
-      <c r="N4" t="str">
+      <c r="Q4" t="str">
         <v>49.99</v>
       </c>
-      <c r="O4" t="str">
+      <c r="R4" t="str">
         <v>25</v>
       </c>
-      <c r="P4" t="str">
-        <v/>
-      </c>
-      <c r="Q4" t="str">
-        <v/>
-      </c>
-      <c r="R4" t="str">
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
         <v>Color</v>
       </c>
-      <c r="S4" t="str">
+      <c r="V4" t="str">
         <v>Red</v>
       </c>
-      <c r="T4" t="str">
+      <c r="W4" t="str">
         <v>Size</v>
       </c>
-      <c r="U4" t="str">
+      <c r="X4" t="str">
         <v>M</v>
       </c>
-      <c r="V4" t="str">
-        <v/>
-      </c>
-      <c r="W4" t="str">
-        <v/>
-      </c>
-      <c r="X4" t="str">
-        <v/>
-      </c>
       <c r="Y4" t="str">
         <v/>
       </c>
       <c r="Z4" t="str">
+        <v/>
+      </c>
+      <c r="AA4" t="str">
+        <v/>
+      </c>
+      <c r="AB4" t="str">
+        <v/>
+      </c>
+      <c r="AC4" t="str">
         <v>0.6</v>
       </c>
-      <c r="AA4" t="str">
-        <v/>
-      </c>
-      <c r="AB4" t="str">
-        <v/>
-      </c>
-      <c r="AC4" t="str">
+      <c r="AD4" t="str">
+        <v/>
+      </c>
+      <c r="AE4" t="str">
+        <v/>
+      </c>
+      <c r="AF4" t="str">
         <v/>
       </c>
     </row>
@@ -788,76 +821,85 @@
         <v/>
       </c>
       <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
         <v>published</v>
       </c>
-      <c r="K5" t="str">
-        <v/>
-      </c>
-      <c r="L5" t="str">
-        <v/>
-      </c>
-      <c r="M5" t="str">
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
         <v>59.99</v>
       </c>
-      <c r="N5" t="str">
-        <v/>
-      </c>
-      <c r="O5" t="str">
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
         <v>10</v>
       </c>
-      <c r="P5" t="str">
+      <c r="S5" t="str">
         <v>https://cdn.example.com/hd-100-blu-l.jpg</v>
       </c>
-      <c r="Q5" t="str">
-        <v/>
-      </c>
-      <c r="R5" t="str">
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
         <v>Color</v>
       </c>
-      <c r="S5" t="str">
+      <c r="V5" t="str">
         <v>Blue</v>
       </c>
-      <c r="T5" t="str">
+      <c r="W5" t="str">
         <v>Size</v>
       </c>
-      <c r="U5" t="str">
+      <c r="X5" t="str">
         <v>L</v>
       </c>
-      <c r="V5" t="str">
-        <v/>
-      </c>
-      <c r="W5" t="str">
-        <v/>
-      </c>
-      <c r="X5" t="str">
-        <v/>
-      </c>
       <c r="Y5" t="str">
         <v/>
       </c>
       <c r="Z5" t="str">
+        <v/>
+      </c>
+      <c r="AA5" t="str">
+        <v/>
+      </c>
+      <c r="AB5" t="str">
+        <v/>
+      </c>
+      <c r="AC5" t="str">
         <v>0.6</v>
       </c>
-      <c r="AA5" t="str">
-        <v/>
-      </c>
-      <c r="AB5" t="str">
-        <v/>
-      </c>
-      <c r="AC5" t="str">
+      <c r="AD5" t="str">
+        <v/>
+      </c>
+      <c r="AE5" t="str">
+        <v/>
+      </c>
+      <c r="AF5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AC5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AF5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B26"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -919,78 +961,98 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>8. Variation rows: use featured_image for per-variation image URL for now.</v>
+        <v>8. Variation rows: use featured_image for per-variation image URL (stored on variations[].image).</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>9. category, brand, unit_type: matched by name/path during import (must exist in catalog).</v>
+        <v>9. Featured and gallery image URLs are linked to Media Library records during import.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>10. seo_title and seo_description: included for future use; not saved until schema supports SEO.</v>
+        <v>10. category, main_category/sub_category/child_category, brand, unit_type: resolved on import.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>11. Upload/import processing is coming in a future release — templates are samples only.</v>
+        <v>11. seo_title and seo_description: included for future use; not saved until schema supports SEO.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v/>
+        <v>12. Product import is live — use Product Imports in the admin or the import API.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Required summary by product_type</v>
+        <v>13. Workflow: upload file → preview with column mapping → review validation → commit.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>simple</v>
-      </c>
-      <c r="B18" t="str">
-        <v>product_type, product_name, sku, price, category (validation-required)</v>
+        <v>14. CSV and XLSX templates are generated from this schema; download either format before filling data.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>variable</v>
-      </c>
-      <c r="B19" t="str">
-        <v>product_type, product_name, sku</v>
+        <v>15. Each import run is recorded in import history; failed rows can be downloaded as an error CSV.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>variation</v>
-      </c>
-      <c r="B20" t="str">
-        <v>product_type, parent_sku, product_name, sku, price, attribute values</v>
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v/>
+        <v>Required summary by product_type</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
+        <v>simple</v>
+      </c>
+      <c r="B22" t="str">
+        <v>product_type, product_name, sku, price, category (validation-required)</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>variable</v>
+      </c>
+      <c r="B23" t="str">
+        <v>product_type, product_name, sku</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>variation</v>
+      </c>
+      <c r="B24" t="str">
+        <v>product_type, parent_sku, product_name, sku, price, attribute values</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
         <v>Source of truth: backend/src/config/productImportSchema.js</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B26"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I33"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1226,10 +1288,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>brand</v>
+        <v>main_category</v>
       </c>
       <c r="B9" t="str">
-        <v>Brand</v>
+        <v>Main Category</v>
       </c>
       <c r="C9" t="str">
         <v>optional</v>
@@ -1241,24 +1303,24 @@
         <v>string</v>
       </c>
       <c r="F9" t="str">
-        <v>Name matching an existing brand</v>
+        <v>Main category name</v>
       </c>
       <c r="G9" t="str">
-        <v>brand</v>
+        <v>category</v>
       </c>
       <c r="H9" t="str">
-        <v>Brand name; resolved to Brand ObjectId on import.</v>
+        <v>Top-level category name (parent null). Used with Sub Category and Child Category.</v>
       </c>
       <c r="I9" t="str">
-        <v>Acme Brand</v>
+        <v>Fashion</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>unit_type</v>
+        <v>sub_category</v>
       </c>
       <c r="B10" t="str">
-        <v>Unit Type</v>
+        <v>Sub Category</v>
       </c>
       <c r="C10" t="str">
         <v>optional</v>
@@ -1270,53 +1332,50 @@
         <v>string</v>
       </c>
       <c r="F10" t="str">
-        <v>Name matching an existing unit type</v>
+        <v>Subcategory name</v>
       </c>
       <c r="G10" t="str">
-        <v>unitType</v>
+        <v>category</v>
       </c>
       <c r="H10" t="str">
-        <v>Unit of measure name; resolved to UnitType ObjectId on import.</v>
+        <v>Second-level category under Main Category.</v>
       </c>
       <c r="I10" t="str">
-        <v>piece</v>
+        <v>Men</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>status</v>
+        <v>child_category</v>
       </c>
       <c r="B11" t="str">
-        <v>Status</v>
+        <v>Child Category</v>
       </c>
       <c r="C11" t="str">
         <v>optional</v>
       </c>
       <c r="D11" t="str">
-        <v>all</v>
+        <v>simple, variable</v>
       </c>
       <c r="E11" t="str">
-        <v>enum</v>
+        <v>string</v>
       </c>
       <c r="F11" t="str">
-        <v>draft, published, inactive</v>
+        <v>Child category name</v>
       </c>
       <c r="G11" t="str">
-        <v>status</v>
+        <v>category</v>
       </c>
       <c r="H11" t="str">
-        <v>Product listing status. Variation rows may set status; importer maps variation rows to variations[].status when supported.</v>
+        <v>Deepest category level; product is assigned here when provided.</v>
       </c>
       <c r="I11" t="str">
-        <v>published</v>
+        <v>T-Shirts</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="str">
-        <v>short_description</v>
-      </c>
       <c r="B12" t="str">
-        <v>Short Description</v>
+        <v>Brand</v>
       </c>
       <c r="C12" t="str">
         <v>optional</v>
@@ -1325,27 +1384,27 @@
         <v>simple, variable</v>
       </c>
       <c r="E12" t="str">
-        <v>text</v>
+        <v>string</v>
       </c>
       <c r="F12" t="str">
-        <v>Plain text or safe HTML</v>
+        <v>Name matching an existing brand</v>
       </c>
       <c r="G12" t="str">
-        <v>shortDescription</v>
+        <v>brand</v>
       </c>
       <c r="H12" t="str">
-        <v>Brief plain text or safe HTML summary.</v>
+        <v>Brand name; resolved to Brand ObjectId on import.</v>
       </c>
       <c r="I12" t="str">
-        <v>Soft cotton everyday tee.</v>
+        <v>Acme Brand</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>description</v>
+        <v>unit_type</v>
       </c>
       <c r="B13" t="str">
-        <v>Description</v>
+        <v>Unit Type</v>
       </c>
       <c r="C13" t="str">
         <v>optional</v>
@@ -1354,491 +1413,491 @@
         <v>simple, variable</v>
       </c>
       <c r="E13" t="str">
-        <v>text</v>
+        <v>string</v>
       </c>
       <c r="F13" t="str">
-        <v>Plain text or safe HTML</v>
+        <v>Name matching an existing unit type</v>
       </c>
       <c r="G13" t="str">
-        <v>description</v>
+        <v>unitType</v>
       </c>
       <c r="H13" t="str">
-        <v>Full product description (plain text or safe HTML).</v>
+        <v>Unit of measure name; resolved to UnitType ObjectId on import.</v>
       </c>
       <c r="I13" t="str">
-        <v>Comfortable crew neck tee for daily wear.</v>
+        <v>piece</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>price</v>
+        <v>status</v>
       </c>
       <c r="B14" t="str">
-        <v>Price</v>
+        <v>Status</v>
       </c>
       <c r="C14" t="str">
-        <v>conditional</v>
+        <v>optional</v>
       </c>
       <c r="D14" t="str">
-        <v>simple, variation (optional on variable parent)</v>
+        <v>all</v>
       </c>
       <c r="E14" t="str">
-        <v>number</v>
+        <v>enum</v>
       </c>
       <c r="F14" t="str">
-        <v>Decimal &gt;= 0</v>
+        <v>draft, published, inactive</v>
       </c>
       <c r="G14" t="str">
-        <v>price</v>
+        <v>status</v>
       </c>
       <c r="H14" t="str">
-        <v>Base price. Required on simple and variation rows; optional on variable parent.</v>
+        <v>Product listing status. Variation rows may set status; importer maps variation rows to variations[].status when supported.</v>
       </c>
       <c r="I14" t="str">
-        <v>29.99</v>
+        <v>published</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>sale_price</v>
+        <v>short_description</v>
       </c>
       <c r="B15" t="str">
-        <v>Sale Price</v>
+        <v>Short Description</v>
       </c>
       <c r="C15" t="str">
         <v>optional</v>
       </c>
       <c r="D15" t="str">
-        <v>simple, variation</v>
+        <v>simple, variable</v>
       </c>
       <c r="E15" t="str">
-        <v>number</v>
+        <v>text</v>
       </c>
       <c r="F15" t="str">
-        <v>Decimal &gt;= 0</v>
+        <v>Plain text or safe HTML</v>
       </c>
       <c r="G15" t="str">
-        <v>salePrice</v>
+        <v>shortDescription</v>
       </c>
       <c r="H15" t="str">
-        <v>Discounted price; must be &lt;= price when set.</v>
+        <v>Brief plain text or safe HTML summary.</v>
       </c>
       <c r="I15" t="str">
-        <v>24.99</v>
+        <v>Soft cotton everyday tee.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>stock</v>
+        <v>description</v>
       </c>
       <c r="B16" t="str">
-        <v>Stock</v>
+        <v>Description</v>
       </c>
       <c r="C16" t="str">
         <v>optional</v>
       </c>
       <c r="D16" t="str">
-        <v>simple, variation</v>
+        <v>simple, variable</v>
       </c>
       <c r="E16" t="str">
-        <v>integer</v>
+        <v>text</v>
       </c>
       <c r="F16" t="str">
-        <v>Integer &gt;= 0</v>
+        <v>Plain text or safe HTML</v>
       </c>
       <c r="G16" t="str">
-        <v>quantity</v>
+        <v>description</v>
       </c>
       <c r="H16" t="str">
-        <v>Inventory quantity. Maps to Product.quantity or variations[].quantity.</v>
+        <v>Full product description (plain text or safe HTML).</v>
       </c>
       <c r="I16" t="str">
-        <v>100</v>
+        <v>Comfortable crew neck tee for daily wear.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>featured_image</v>
+        <v>price</v>
       </c>
       <c r="B17" t="str">
-        <v>Featured Image</v>
+        <v>Price</v>
       </c>
       <c r="C17" t="str">
-        <v>optional</v>
+        <v>conditional</v>
       </c>
       <c r="D17" t="str">
-        <v>simple, variable, variation</v>
+        <v>simple, variation (optional on variable parent)</v>
       </c>
       <c r="E17" t="str">
-        <v>url</v>
+        <v>number</v>
       </c>
       <c r="F17" t="str">
-        <v>http(s) URL or server path</v>
+        <v>Decimal &gt;= 0</v>
       </c>
       <c r="G17" t="str">
-        <v>featuredImage</v>
+        <v>price</v>
       </c>
       <c r="H17" t="str">
-        <v>Primary image URL. On variation rows, use as variation image (maps to variations[].image) until a dedicated column exists.</v>
+        <v>Base price. Required on simple and variation rows; optional on variable parent.</v>
       </c>
       <c r="I17" t="str">
-        <v>https://cdn.example.com/tee-001.jpg</v>
+        <v>29.99</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>gallery_images</v>
+        <v>sale_price</v>
       </c>
       <c r="B18" t="str">
-        <v>Gallery Images</v>
+        <v>Sale Price</v>
       </c>
       <c r="C18" t="str">
         <v>optional</v>
       </c>
       <c r="D18" t="str">
-        <v>simple, variable</v>
+        <v>simple, variation</v>
       </c>
       <c r="E18" t="str">
-        <v>string</v>
+        <v>number</v>
       </c>
       <c r="F18" t="str">
-        <v>Pipe-separated URLs</v>
+        <v>Decimal &gt;= 0</v>
       </c>
       <c r="G18" t="str">
-        <v>galleryImages</v>
+        <v>salePrice</v>
       </c>
       <c r="H18" t="str">
-        <v>Multiple image URLs separated by pipe (|). Comma used only if no pipe present.</v>
+        <v>Discounted price; must be &lt;= price when set.</v>
       </c>
       <c r="I18" t="str">
-        <v>https://cdn.example.com/a.jpg|https://cdn.example.com/b.jpg</v>
+        <v>24.99</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>attribute_1_name</v>
+        <v>stock</v>
       </c>
       <c r="B19" t="str">
-        <v>Attribute 1 Name</v>
+        <v>Stock</v>
       </c>
       <c r="C19" t="str">
-        <v>conditional</v>
+        <v>optional</v>
       </c>
       <c r="D19" t="str">
-        <v>variable (name), variation (value)</v>
+        <v>simple, variation</v>
       </c>
       <c r="E19" t="str">
-        <v>string</v>
+        <v>integer</v>
       </c>
       <c r="F19" t="str">
-        <v>Catalog attribute name</v>
+        <v>Integer &gt;= 0</v>
       </c>
       <c r="G19" t="str">
-        <v>attributes[].name</v>
+        <v>quantity</v>
       </c>
       <c r="H19" t="str">
-        <v>First variation attribute label on variable parent; value on variation rows.</v>
+        <v>Inventory quantity. Maps to Product.quantity or variations[].quantity.</v>
       </c>
       <c r="I19" t="str">
-        <v>Color</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>attribute_1_value</v>
+        <v>featured_image</v>
       </c>
       <c r="B20" t="str">
-        <v>Attribute 1 Value</v>
+        <v>Featured Image</v>
       </c>
       <c r="C20" t="str">
-        <v>conditional</v>
+        <v>optional</v>
       </c>
       <c r="D20" t="str">
-        <v>variation</v>
+        <v>simple, variable, variation</v>
       </c>
       <c r="E20" t="str">
-        <v>string</v>
+        <v>url</v>
       </c>
       <c r="F20" t="str">
-        <v>Defined attribute value</v>
+        <v>http(s) URL or server path</v>
       </c>
       <c r="G20" t="str">
-        <v>variations[].attributes[].value</v>
+        <v>featuredImage</v>
       </c>
       <c r="H20" t="str">
-        <v>Value for attribute 1 on variation rows.</v>
+        <v>Primary image URL or server path. On import, linked to a Media Library record (featuredMediaId) while keeping the URL on the product.</v>
       </c>
       <c r="I20" t="str">
-        <v>Red</v>
+        <v>https://cdn.example.com/tee-001.jpg</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>attribute_2_name</v>
+        <v>gallery_images</v>
       </c>
       <c r="B21" t="str">
-        <v>Attribute 2 Name</v>
+        <v>Gallery Images</v>
       </c>
       <c r="C21" t="str">
         <v>optional</v>
       </c>
       <c r="D21" t="str">
-        <v>variable (name), variation (value)</v>
+        <v>simple, variable</v>
       </c>
       <c r="E21" t="str">
         <v>string</v>
       </c>
       <c r="F21" t="str">
-        <v>Catalog attribute name</v>
+        <v>Pipe-separated URLs</v>
       </c>
       <c r="G21" t="str">
-        <v>attributes[].name</v>
+        <v>galleryImages</v>
       </c>
       <c r="H21" t="str">
-        <v>Second variation attribute label on variable parent.</v>
+        <v>Multiple image URLs separated by pipe (|). Each URL is linked to Media Library records on import.</v>
       </c>
       <c r="I21" t="str">
-        <v>Size</v>
+        <v>https://cdn.example.com/a.jpg|https://cdn.example.com/b.jpg</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>attribute_2_value</v>
+        <v>attribute_1_name</v>
       </c>
       <c r="B22" t="str">
-        <v>Attribute 2 Value</v>
+        <v>Attribute 1 Name</v>
       </c>
       <c r="C22" t="str">
-        <v>optional</v>
+        <v>conditional</v>
       </c>
       <c r="D22" t="str">
-        <v>variation</v>
+        <v>variable (name), variation (value)</v>
       </c>
       <c r="E22" t="str">
         <v>string</v>
       </c>
       <c r="F22" t="str">
-        <v>Defined attribute value</v>
+        <v>Catalog attribute name</v>
       </c>
       <c r="G22" t="str">
-        <v>variations[].attributes[].value</v>
+        <v>attributes[].name</v>
       </c>
       <c r="H22" t="str">
-        <v>Value for attribute 2 on variation rows.</v>
+        <v>First variation attribute label on variable parent; value on variation rows.</v>
       </c>
       <c r="I22" t="str">
-        <v>M</v>
+        <v>Color</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>variation_options</v>
+        <v>attribute_1_value</v>
       </c>
       <c r="B23" t="str">
-        <v>Variation Options</v>
+        <v>Attribute 1 Value</v>
       </c>
       <c r="C23" t="str">
-        <v>optional</v>
+        <v>conditional</v>
       </c>
       <c r="D23" t="str">
-        <v>variable</v>
+        <v>variation</v>
       </c>
       <c r="E23" t="str">
         <v>string</v>
       </c>
       <c r="F23" t="str">
-        <v>Semicolon-separated names</v>
+        <v>Defined attribute value</v>
       </c>
       <c r="G23" t="str">
-        <v/>
+        <v>variations[].attributes[].value</v>
       </c>
       <c r="H23" t="str">
-        <v>Variation axes on variable parent; semicolon-separated attribute names.</v>
+        <v>Value for attribute 1 on variation rows.</v>
       </c>
       <c r="I23" t="str">
-        <v>Color;Size</v>
+        <v>Red</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>seo_title</v>
+        <v>attribute_2_name</v>
       </c>
       <c r="B24" t="str">
-        <v>SEO Title</v>
+        <v>Attribute 2 Name</v>
       </c>
       <c r="C24" t="str">
         <v>optional</v>
       </c>
       <c r="D24" t="str">
-        <v>simple, variable</v>
+        <v>variable (name), variation (value)</v>
       </c>
       <c r="E24" t="str">
         <v>string</v>
       </c>
       <c r="F24" t="str">
-        <v>Any text</v>
+        <v>Catalog attribute name</v>
       </c>
       <c r="G24" t="str">
-        <v/>
+        <v>attributes[].name</v>
       </c>
       <c r="H24" t="str">
-        <v>Future SEO field; ignored by importer until Product schema supports it.</v>
+        <v>Second variation attribute label on variable parent.</v>
       </c>
       <c r="I24" t="str">
-        <v>Classic Cotton Tee | Acme Store</v>
+        <v>Size</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>seo_description</v>
+        <v>attribute_2_value</v>
       </c>
       <c r="B25" t="str">
-        <v>SEO Description</v>
+        <v>Attribute 2 Value</v>
       </c>
       <c r="C25" t="str">
         <v>optional</v>
       </c>
       <c r="D25" t="str">
-        <v>simple, variable</v>
+        <v>variation</v>
       </c>
       <c r="E25" t="str">
         <v>string</v>
       </c>
       <c r="F25" t="str">
-        <v>Any text</v>
+        <v>Defined attribute value</v>
       </c>
       <c r="G25" t="str">
-        <v/>
+        <v>variations[].attributes[].value</v>
       </c>
       <c r="H25" t="str">
-        <v>Future SEO field; ignored by importer until Product schema supports it.</v>
+        <v>Value for attribute 2 on variation rows.</v>
       </c>
       <c r="I25" t="str">
-        <v>Shop our classic cotton tee.</v>
+        <v>M</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>tags</v>
+        <v>variation_options</v>
       </c>
       <c r="B26" t="str">
-        <v>Tags</v>
+        <v>Variation Options</v>
       </c>
       <c r="C26" t="str">
         <v>optional</v>
       </c>
       <c r="D26" t="str">
-        <v>simple, variable</v>
+        <v>variable</v>
       </c>
       <c r="E26" t="str">
         <v>string</v>
       </c>
       <c r="F26" t="str">
-        <v>Comma-separated values</v>
+        <v>Semicolon-separated names</v>
       </c>
       <c r="G26" t="str">
         <v/>
       </c>
       <c r="H26" t="str">
-        <v>Comma-separated tags for future catalog features.</v>
+        <v>Variation axes on variable parent; semicolon-separated attribute names.</v>
       </c>
       <c r="I26" t="str">
-        <v>tee,cotton,basics</v>
+        <v>Color;Size</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>weight</v>
+        <v>seo_title</v>
       </c>
       <c r="B27" t="str">
-        <v>Weight</v>
+        <v>SEO Title</v>
       </c>
       <c r="C27" t="str">
         <v>optional</v>
       </c>
       <c r="D27" t="str">
-        <v>all</v>
+        <v>simple, variable</v>
       </c>
       <c r="E27" t="str">
-        <v>number</v>
+        <v>string</v>
       </c>
       <c r="F27" t="str">
-        <v>Decimal &gt;= 0</v>
+        <v>Any text</v>
       </c>
       <c r="G27" t="str">
         <v/>
       </c>
       <c r="H27" t="str">
-        <v>Product weight for future shipping calculations.</v>
+        <v>Future SEO field; ignored by importer until Product schema supports it.</v>
       </c>
       <c r="I27" t="str">
-        <v>0.25</v>
+        <v>Classic Cotton Tee | Acme Store</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>length</v>
+        <v>seo_description</v>
       </c>
       <c r="B28" t="str">
-        <v>Length</v>
+        <v>SEO Description</v>
       </c>
       <c r="C28" t="str">
         <v>optional</v>
       </c>
       <c r="D28" t="str">
-        <v>all</v>
+        <v>simple, variable</v>
       </c>
       <c r="E28" t="str">
-        <v>number</v>
+        <v>string</v>
       </c>
       <c r="F28" t="str">
-        <v>Decimal &gt;= 0</v>
+        <v>Any text</v>
       </c>
       <c r="G28" t="str">
         <v/>
       </c>
       <c r="H28" t="str">
-        <v>Package length for future shipping.</v>
+        <v>Future SEO field; ignored by importer until Product schema supports it.</v>
       </c>
       <c r="I28" t="str">
-        <v>30</v>
+        <v>Shop our classic cotton tee.</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>width</v>
+        <v>tags</v>
       </c>
       <c r="B29" t="str">
-        <v>Width</v>
+        <v>Tags</v>
       </c>
       <c r="C29" t="str">
         <v>optional</v>
       </c>
       <c r="D29" t="str">
-        <v>all</v>
+        <v>simple, variable</v>
       </c>
       <c r="E29" t="str">
-        <v>number</v>
+        <v>string</v>
       </c>
       <c r="F29" t="str">
-        <v>Decimal &gt;= 0</v>
+        <v>Comma-separated values</v>
       </c>
       <c r="G29" t="str">
         <v/>
       </c>
       <c r="H29" t="str">
-        <v>Package width for future shipping.</v>
+        <v>Comma-separated tags for future catalog features.</v>
       </c>
       <c r="I29" t="str">
-        <v>25</v>
+        <v>tee,cotton,basics</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>height</v>
+        <v>weight</v>
       </c>
       <c r="B30" t="str">
-        <v>Height</v>
+        <v>Weight</v>
       </c>
       <c r="C30" t="str">
         <v>optional</v>
@@ -1856,22 +1915,109 @@
         <v/>
       </c>
       <c r="H30" t="str">
+        <v>Product weight for future shipping calculations.</v>
+      </c>
+      <c r="I30" t="str">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>length</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Length</v>
+      </c>
+      <c r="C31" t="str">
+        <v>optional</v>
+      </c>
+      <c r="D31" t="str">
+        <v>all</v>
+      </c>
+      <c r="E31" t="str">
+        <v>number</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Decimal &gt;= 0</v>
+      </c>
+      <c r="G31" t="str">
+        <v/>
+      </c>
+      <c r="H31" t="str">
+        <v>Package length for future shipping.</v>
+      </c>
+      <c r="I31" t="str">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>width</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Width</v>
+      </c>
+      <c r="C32" t="str">
+        <v>optional</v>
+      </c>
+      <c r="D32" t="str">
+        <v>all</v>
+      </c>
+      <c r="E32" t="str">
+        <v>number</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Decimal &gt;= 0</v>
+      </c>
+      <c r="G32" t="str">
+        <v/>
+      </c>
+      <c r="H32" t="str">
+        <v>Package width for future shipping.</v>
+      </c>
+      <c r="I32" t="str">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>height</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Height</v>
+      </c>
+      <c r="C33" t="str">
+        <v>optional</v>
+      </c>
+      <c r="D33" t="str">
+        <v>all</v>
+      </c>
+      <c r="E33" t="str">
+        <v>number</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Decimal &gt;= 0</v>
+      </c>
+      <c r="G33" t="str">
+        <v/>
+      </c>
+      <c r="H33" t="str">
         <v>Package height for future shipping.</v>
       </c>
-      <c r="I30" t="str">
+      <c r="I33" t="str">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I33"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC2"/>
+  <dimension ref="A1:AF2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1896,69 +2042,75 @@
         <v>category</v>
       </c>
       <c r="H1" t="str">
-        <v>brand</v>
+        <v>main_category</v>
       </c>
       <c r="I1" t="str">
+        <v>sub_category</v>
+      </c>
+      <c r="J1" t="str">
+        <v>child_category</v>
+      </c>
+      <c r="L1" t="str">
         <v>unit_type</v>
       </c>
-      <c r="J1" t="str">
+      <c r="M1" t="str">
         <v>status</v>
       </c>
-      <c r="K1" t="str">
+      <c r="N1" t="str">
         <v>short_description</v>
       </c>
-      <c r="L1" t="str">
+      <c r="O1" t="str">
         <v>description</v>
       </c>
-      <c r="M1" t="str">
+      <c r="P1" t="str">
         <v>price</v>
       </c>
-      <c r="N1" t="str">
+      <c r="Q1" t="str">
         <v>sale_price</v>
       </c>
-      <c r="O1" t="str">
+      <c r="R1" t="str">
         <v>stock</v>
       </c>
-      <c r="P1" t="str">
+      <c r="S1" t="str">
         <v>featured_image</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="T1" t="str">
         <v>gallery_images</v>
       </c>
-      <c r="R1" t="str">
+      <c r="U1" t="str">
         <v>attribute_1_name</v>
       </c>
-      <c r="S1" t="str">
+      <c r="V1" t="str">
         <v>attribute_1_value</v>
       </c>
-      <c r="T1" t="str">
+      <c r="W1" t="str">
         <v>attribute_2_name</v>
       </c>
-      <c r="U1" t="str">
+      <c r="X1" t="str">
         <v>attribute_2_value</v>
       </c>
-      <c r="V1" t="str">
+      <c r="Y1" t="str">
         <v>variation_options</v>
       </c>
-      <c r="W1" t="str">
+      <c r="Z1" t="str">
         <v>seo_title</v>
       </c>
-      <c r="X1" t="str">
+      <c r="AA1" t="str">
         <v>seo_description</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="AB1" t="str">
         <v>tags</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AC1" t="str">
         <v>weight</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AD1" t="str">
         <v>length</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AE1" t="str">
         <v>width</v>
       </c>
-      <c r="AC1" t="str">
+      <c r="AF1" t="str">
         <v>height</v>
       </c>
     </row>
@@ -1985,44 +2137,44 @@
         <v>Apparel &gt; Tees</v>
       </c>
       <c r="H2" t="str">
-        <v>Acme Brand</v>
+        <v/>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
         <v>piece</v>
       </c>
-      <c r="J2" t="str">
+      <c r="M2" t="str">
         <v>published</v>
       </c>
-      <c r="K2" t="str">
+      <c r="N2" t="str">
         <v>Soft cotton everyday tee.</v>
       </c>
-      <c r="L2" t="str">
+      <c r="O2" t="str">
         <v>Comfortable crew neck tee for daily wear.</v>
       </c>
-      <c r="M2" t="str">
+      <c r="P2" t="str">
         <v>29.99</v>
       </c>
-      <c r="N2" t="str">
+      <c r="Q2" t="str">
         <v>24.99</v>
       </c>
-      <c r="O2" t="str">
+      <c r="R2" t="str">
         <v>100</v>
       </c>
-      <c r="P2" t="str">
+      <c r="S2" t="str">
         <v>https://cdn.example.com/tee-001.jpg</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="T2" t="str">
         <v>https://cdn.example.com/tee-001-a.jpg|https://cdn.example.com/tee-001-b.jpg</v>
       </c>
-      <c r="R2" t="str">
-        <v/>
-      </c>
-      <c r="S2" t="str">
-        <v/>
-      </c>
-      <c r="T2" t="str">
-        <v/>
-      </c>
       <c r="U2" t="str">
         <v/>
       </c>
@@ -2030,37 +2182,46 @@
         <v/>
       </c>
       <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
+        <v/>
+      </c>
+      <c r="Z2" t="str">
         <v>Classic Cotton Tee | Acme Store</v>
       </c>
-      <c r="X2" t="str">
+      <c r="AA2" t="str">
         <v>Shop our classic cotton tee.</v>
       </c>
-      <c r="Y2" t="str">
+      <c r="AB2" t="str">
         <v>tee,cotton,basics</v>
       </c>
-      <c r="Z2" t="str">
+      <c r="AC2" t="str">
         <v>0.25</v>
       </c>
-      <c r="AA2" t="str">
+      <c r="AD2" t="str">
         <v>30</v>
       </c>
-      <c r="AB2" t="str">
+      <c r="AE2" t="str">
         <v>25</v>
       </c>
-      <c r="AC2" t="str">
+      <c r="AF2" t="str">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AC2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AF2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC4"/>
+  <dimension ref="A1:AF4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2085,69 +2246,75 @@
         <v>category</v>
       </c>
       <c r="H1" t="str">
-        <v>brand</v>
+        <v>main_category</v>
       </c>
       <c r="I1" t="str">
+        <v>sub_category</v>
+      </c>
+      <c r="J1" t="str">
+        <v>child_category</v>
+      </c>
+      <c r="L1" t="str">
         <v>unit_type</v>
       </c>
-      <c r="J1" t="str">
+      <c r="M1" t="str">
         <v>status</v>
       </c>
-      <c r="K1" t="str">
+      <c r="N1" t="str">
         <v>short_description</v>
       </c>
-      <c r="L1" t="str">
+      <c r="O1" t="str">
         <v>description</v>
       </c>
-      <c r="M1" t="str">
+      <c r="P1" t="str">
         <v>price</v>
       </c>
-      <c r="N1" t="str">
+      <c r="Q1" t="str">
         <v>sale_price</v>
       </c>
-      <c r="O1" t="str">
+      <c r="R1" t="str">
         <v>stock</v>
       </c>
-      <c r="P1" t="str">
+      <c r="S1" t="str">
         <v>featured_image</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="T1" t="str">
         <v>gallery_images</v>
       </c>
-      <c r="R1" t="str">
+      <c r="U1" t="str">
         <v>attribute_1_name</v>
       </c>
-      <c r="S1" t="str">
+      <c r="V1" t="str">
         <v>attribute_1_value</v>
       </c>
-      <c r="T1" t="str">
+      <c r="W1" t="str">
         <v>attribute_2_name</v>
       </c>
-      <c r="U1" t="str">
+      <c r="X1" t="str">
         <v>attribute_2_value</v>
       </c>
-      <c r="V1" t="str">
+      <c r="Y1" t="str">
         <v>variation_options</v>
       </c>
-      <c r="W1" t="str">
+      <c r="Z1" t="str">
         <v>seo_title</v>
       </c>
-      <c r="X1" t="str">
+      <c r="AA1" t="str">
         <v>seo_description</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="AB1" t="str">
         <v>tags</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AC1" t="str">
         <v>weight</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AD1" t="str">
         <v>length</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AE1" t="str">
         <v>width</v>
       </c>
-      <c r="AC1" t="str">
+      <c r="AF1" t="str">
         <v>height</v>
       </c>
     </row>
@@ -2174,69 +2341,78 @@
         <v>Apparel &gt; Hoodies</v>
       </c>
       <c r="H2" t="str">
-        <v>Acme Brand</v>
+        <v/>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
         <v>piece</v>
       </c>
-      <c r="J2" t="str">
+      <c r="M2" t="str">
         <v>published</v>
       </c>
-      <c r="K2" t="str">
+      <c r="N2" t="str">
         <v>Warm layered hoodie.</v>
       </c>
-      <c r="L2" t="str">
+      <c r="O2" t="str">
         <v>Premium fleece hoodie with kangaroo pocket.</v>
       </c>
-      <c r="M2" t="str">
+      <c r="P2" t="str">
         <v>59.99</v>
       </c>
-      <c r="N2" t="str">
-        <v/>
-      </c>
-      <c r="O2" t="str">
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
         <v>0</v>
       </c>
-      <c r="P2" t="str">
+      <c r="S2" t="str">
         <v>https://cdn.example.com/hd-100.jpg</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="T2" t="str">
         <v>https://cdn.example.com/hd-100-alt.jpg</v>
       </c>
-      <c r="R2" t="str">
+      <c r="U2" t="str">
         <v>Color</v>
       </c>
-      <c r="S2" t="str">
-        <v/>
-      </c>
-      <c r="T2" t="str">
+      <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
         <v>Size</v>
       </c>
-      <c r="U2" t="str">
-        <v/>
-      </c>
-      <c r="V2" t="str">
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
         <v>Color;Size</v>
       </c>
-      <c r="W2" t="str">
+      <c r="Z2" t="str">
         <v>Hooded Sweatshirt</v>
       </c>
-      <c r="X2" t="str">
+      <c r="AA2" t="str">
         <v>Variable product parent row.</v>
       </c>
-      <c r="Y2" t="str">
+      <c r="AB2" t="str">
         <v>hoodie,apparel</v>
       </c>
-      <c r="Z2" t="str">
-        <v/>
-      </c>
-      <c r="AA2" t="str">
-        <v/>
-      </c>
-      <c r="AB2" t="str">
-        <v/>
-      </c>
       <c r="AC2" t="str">
+        <v/>
+      </c>
+      <c r="AD2" t="str">
+        <v/>
+      </c>
+      <c r="AE2" t="str">
+        <v/>
+      </c>
+      <c r="AF2" t="str">
         <v/>
       </c>
     </row>
@@ -2269,63 +2445,72 @@
         <v/>
       </c>
       <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
         <v>published</v>
       </c>
-      <c r="K3" t="str">
-        <v/>
-      </c>
-      <c r="L3" t="str">
-        <v/>
-      </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
         <v>59.99</v>
       </c>
-      <c r="N3" t="str">
+      <c r="Q3" t="str">
         <v>49.99</v>
       </c>
-      <c r="O3" t="str">
+      <c r="R3" t="str">
         <v>25</v>
       </c>
-      <c r="P3" t="str">
-        <v/>
-      </c>
-      <c r="Q3" t="str">
-        <v/>
-      </c>
-      <c r="R3" t="str">
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
         <v>Color</v>
       </c>
-      <c r="S3" t="str">
+      <c r="V3" t="str">
         <v>Red</v>
       </c>
-      <c r="T3" t="str">
+      <c r="W3" t="str">
         <v>Size</v>
       </c>
-      <c r="U3" t="str">
+      <c r="X3" t="str">
         <v>M</v>
       </c>
-      <c r="V3" t="str">
-        <v/>
-      </c>
-      <c r="W3" t="str">
-        <v/>
-      </c>
-      <c r="X3" t="str">
-        <v/>
-      </c>
       <c r="Y3" t="str">
         <v/>
       </c>
       <c r="Z3" t="str">
+        <v/>
+      </c>
+      <c r="AA3" t="str">
+        <v/>
+      </c>
+      <c r="AB3" t="str">
+        <v/>
+      </c>
+      <c r="AC3" t="str">
         <v>0.6</v>
       </c>
-      <c r="AA3" t="str">
-        <v/>
-      </c>
-      <c r="AB3" t="str">
-        <v/>
-      </c>
-      <c r="AC3" t="str">
+      <c r="AD3" t="str">
+        <v/>
+      </c>
+      <c r="AE3" t="str">
+        <v/>
+      </c>
+      <c r="AF3" t="str">
         <v/>
       </c>
     </row>
@@ -2358,69 +2543,78 @@
         <v/>
       </c>
       <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
         <v>published</v>
       </c>
-      <c r="K4" t="str">
-        <v/>
-      </c>
-      <c r="L4" t="str">
-        <v/>
-      </c>
-      <c r="M4" t="str">
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
         <v>59.99</v>
       </c>
-      <c r="N4" t="str">
-        <v/>
-      </c>
-      <c r="O4" t="str">
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
         <v>10</v>
       </c>
-      <c r="P4" t="str">
+      <c r="S4" t="str">
         <v>https://cdn.example.com/hd-100-blu-l.jpg</v>
       </c>
-      <c r="Q4" t="str">
-        <v/>
-      </c>
-      <c r="R4" t="str">
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
         <v>Color</v>
       </c>
-      <c r="S4" t="str">
+      <c r="V4" t="str">
         <v>Blue</v>
       </c>
-      <c r="T4" t="str">
+      <c r="W4" t="str">
         <v>Size</v>
       </c>
-      <c r="U4" t="str">
+      <c r="X4" t="str">
         <v>L</v>
       </c>
-      <c r="V4" t="str">
-        <v/>
-      </c>
-      <c r="W4" t="str">
-        <v/>
-      </c>
-      <c r="X4" t="str">
-        <v/>
-      </c>
       <c r="Y4" t="str">
         <v/>
       </c>
       <c r="Z4" t="str">
+        <v/>
+      </c>
+      <c r="AA4" t="str">
+        <v/>
+      </c>
+      <c r="AB4" t="str">
+        <v/>
+      </c>
+      <c r="AC4" t="str">
         <v>0.6</v>
       </c>
-      <c r="AA4" t="str">
-        <v/>
-      </c>
-      <c r="AB4" t="str">
-        <v/>
-      </c>
-      <c r="AC4" t="str">
+      <c r="AD4" t="str">
+        <v/>
+      </c>
+      <c r="AE4" t="str">
+        <v/>
+      </c>
+      <c r="AF4" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AC4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AF4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>